<commit_message>
Add results for task 5
</commit_message>
<xml_diff>
--- a/ExperimentSummarySheet_Ex1.xlsx
+++ b/ExperimentSummarySheet_Ex1.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="55">
   <si>
     <t xml:space="preserve">Group Name/Student Name</t>
   </si>
@@ -167,14 +167,33 @@
   </si>
   <si>
     <t xml:space="preserve">As expected best performance on positive and negative class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FinBERT Multiclass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FinBERT Autotokenizer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lr=2e-5, weight_decay=0.001, batch_size = 16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FinBERT Binary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neutral removed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="0.00%"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -250,7 +269,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -260,6 +279,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -386,7 +409,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.51"/>
@@ -465,7 +488,6 @@
       <c r="I2" s="1" t="n">
         <v>0.65</v>
       </c>
-      <c r="J2" s="0"/>
       <c r="K2" s="1" t="s">
         <v>16</v>
       </c>
@@ -498,7 +520,6 @@
       <c r="I3" s="1" t="n">
         <v>0.46</v>
       </c>
-      <c r="J3" s="0"/>
       <c r="K3" s="1" t="s">
         <v>18</v>
       </c>
@@ -531,7 +552,6 @@
       <c r="I4" s="1" t="n">
         <v>0.66</v>
       </c>
-      <c r="J4" s="0"/>
       <c r="K4" s="1" t="s">
         <v>20</v>
       </c>
@@ -564,7 +584,6 @@
       <c r="I5" s="1" t="n">
         <v>0.46</v>
       </c>
-      <c r="J5" s="0"/>
       <c r="K5" s="1" t="s">
         <v>21</v>
       </c>
@@ -597,7 +616,6 @@
       <c r="I6" s="1" t="n">
         <v>0.64</v>
       </c>
-      <c r="J6" s="0"/>
       <c r="K6" s="1" t="s">
         <v>23</v>
       </c>
@@ -630,7 +648,6 @@
       <c r="I7" s="1" t="n">
         <v>0.46</v>
       </c>
-      <c r="J7" s="0"/>
       <c r="K7" s="1" t="s">
         <v>21</v>
       </c>
@@ -663,7 +680,6 @@
       <c r="I8" s="1" t="n">
         <v>0.66</v>
       </c>
-      <c r="J8" s="0"/>
       <c r="K8" s="1" t="s">
         <v>25</v>
       </c>
@@ -696,7 +712,6 @@
       <c r="I9" s="1" t="n">
         <v>0.47</v>
       </c>
-      <c r="J9" s="0"/>
       <c r="K9" s="1" t="s">
         <v>25</v>
       </c>
@@ -729,7 +744,6 @@
       <c r="I10" s="1" t="n">
         <v>0.59</v>
       </c>
-      <c r="J10" s="0"/>
       <c r="K10" s="1" t="s">
         <v>27</v>
       </c>
@@ -762,7 +776,6 @@
       <c r="I11" s="1" t="n">
         <v>0.61</v>
       </c>
-      <c r="J11" s="0"/>
       <c r="K11" s="1" t="s">
         <v>28</v>
       </c>
@@ -795,7 +808,6 @@
       <c r="I12" s="1" t="n">
         <v>0.53</v>
       </c>
-      <c r="J12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
@@ -825,7 +837,6 @@
       <c r="I13" s="1" t="n">
         <v>0.54</v>
       </c>
-      <c r="J13" s="0"/>
       <c r="K13" s="1" t="s">
         <v>30</v>
       </c>
@@ -858,7 +869,6 @@
       <c r="I14" s="1" t="n">
         <v>0.67</v>
       </c>
-      <c r="J14" s="0"/>
       <c r="K14" s="1" t="s">
         <v>33</v>
       </c>
@@ -891,7 +901,6 @@
       <c r="I15" s="1" t="n">
         <v>0.68</v>
       </c>
-      <c r="J15" s="0"/>
       <c r="K15" s="1" t="s">
         <v>34</v>
       </c>
@@ -924,14 +933,10 @@
       <c r="I16" s="1" t="n">
         <v>0.78</v>
       </c>
-      <c r="J16" s="0"/>
       <c r="K16" s="1" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="J17" s="0"/>
-    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>11</v>
@@ -960,7 +965,6 @@
       <c r="I18" s="1" t="n">
         <v>0.7</v>
       </c>
-      <c r="J18" s="0"/>
       <c r="K18" s="1" t="s">
         <v>16</v>
       </c>
@@ -993,7 +997,6 @@
       <c r="I19" s="1" t="n">
         <v>0.7</v>
       </c>
-      <c r="J19" s="0"/>
       <c r="K19" s="1" t="s">
         <v>40</v>
       </c>
@@ -1026,7 +1029,6 @@
       <c r="I20" s="1" t="n">
         <v>0.69</v>
       </c>
-      <c r="J20" s="0"/>
       <c r="K20" s="1" t="s">
         <v>41</v>
       </c>
@@ -1059,7 +1061,6 @@
       <c r="I21" s="1" t="n">
         <v>0.69</v>
       </c>
-      <c r="J21" s="0"/>
       <c r="K21" s="1" t="s">
         <v>41</v>
       </c>
@@ -1092,7 +1093,6 @@
       <c r="I22" s="1" t="n">
         <v>0.69</v>
       </c>
-      <c r="J22" s="0"/>
       <c r="K22" s="1" t="s">
         <v>41</v>
       </c>
@@ -1125,7 +1125,6 @@
       <c r="I23" s="1" t="n">
         <v>0.69</v>
       </c>
-      <c r="J23" s="0"/>
       <c r="K23" s="1" t="s">
         <v>41</v>
       </c>
@@ -1158,7 +1157,6 @@
       <c r="I24" s="1" t="n">
         <v>0.71</v>
       </c>
-      <c r="J24" s="0"/>
       <c r="K24" s="1" t="s">
         <v>41</v>
       </c>
@@ -1191,7 +1189,6 @@
       <c r="I25" s="1" t="n">
         <v>0.7</v>
       </c>
-      <c r="J25" s="0"/>
       <c r="K25" s="1" t="s">
         <v>41</v>
       </c>
@@ -1224,7 +1221,6 @@
       <c r="I26" s="1" t="n">
         <v>0.71</v>
       </c>
-      <c r="J26" s="0"/>
       <c r="K26" s="1" t="s">
         <v>43</v>
       </c>
@@ -1257,7 +1253,6 @@
       <c r="I27" s="1" t="n">
         <v>0.72</v>
       </c>
-      <c r="J27" s="0"/>
       <c r="K27" s="1" t="s">
         <v>43</v>
       </c>
@@ -1290,7 +1285,6 @@
       <c r="I28" s="1" t="n">
         <v>0.68</v>
       </c>
-      <c r="J28" s="0"/>
       <c r="K28" s="1" t="s">
         <v>45</v>
       </c>
@@ -1323,7 +1317,6 @@
       <c r="I29" s="1" t="n">
         <v>0.68</v>
       </c>
-      <c r="J29" s="0"/>
       <c r="K29" s="1" t="s">
         <v>45</v>
       </c>
@@ -1356,9 +1349,66 @@
       <c r="I30" s="1" t="n">
         <v>0.83</v>
       </c>
-      <c r="J30" s="0"/>
       <c r="K30" s="1" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="D32" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="F32" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="G32" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>0.8972</v>
+      </c>
+      <c r="I32" s="0" t="n">
+        <v>0.883</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="D33" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="F33" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="G33" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>0.9723</v>
+      </c>
+      <c r="I33" s="0" t="n">
+        <v>0.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>